<commit_message>
cambios en el INSTITUTO
</commit_message>
<xml_diff>
--- a/Capitulo999_INSTITUTO/Taller2_2026/Taller02_2026_ISGM.xlsx
+++ b/Capitulo999_INSTITUTO/Taller2_2026/Taller02_2026_ISGM.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="35">
   <si>
     <t>Apellido y Nombre</t>
   </si>
@@ -109,6 +109,24 @@
   </si>
   <si>
     <t>Ejercicio 02</t>
+  </si>
+  <si>
+    <t>Ejercicio</t>
+  </si>
+  <si>
+    <t>Evaluación 2</t>
+  </si>
+  <si>
+    <t>24.06.2026</t>
+  </si>
+  <si>
+    <t>10 (Excelente)</t>
+  </si>
+  <si>
+    <t>8 (Excelente)</t>
+  </si>
+  <si>
+    <t>9 (Muy bien)</t>
   </si>
 </sst>
 </file>
@@ -153,7 +171,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -190,6 +208,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -203,11 +227,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -220,11 +249,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -505,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:L14"/>
+  <dimension ref="B1:O14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
@@ -518,28 +546,35 @@
     <col min="9" max="9" width="0" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.85546875" customWidth="1"/>
+    <col min="14" max="14" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="6" t="s">
+    <row r="1" spans="2:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="4" t="s">
+      <c r="C1" s="11"/>
+      <c r="D1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4"/>
-      <c r="G1" s="5" t="s">
+      <c r="E1" s="9"/>
+      <c r="G1" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="5"/>
-      <c r="J1" s="5" t="s">
+      <c r="H1" s="10"/>
+      <c r="J1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-    </row>
-    <row r="2" spans="2:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+    </row>
+    <row r="2" spans="2:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>11</v>
       </c>
@@ -558,21 +593,29 @@
       <c r="H2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-    </row>
-    <row r="3" spans="2:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+    </row>
+    <row r="3" spans="2:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="K3" s="1" t="s">
         <v>27</v>
       </c>
       <c r="L3" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="N3" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>1</v>
       </c>
@@ -591,14 +634,20 @@
       <c r="J4" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>2</v>
       </c>
@@ -617,14 +666,20 @@
       <c r="J5" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="L5" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M5" t="s">
+        <v>24</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>3</v>
       </c>
@@ -646,14 +701,20 @@
       <c r="J6" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" t="s">
+        <v>24</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>4</v>
       </c>
@@ -672,14 +733,20 @@
       <c r="J7" t="s">
         <v>24</v>
       </c>
-      <c r="K7" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="L7" s="10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="M7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
         <v>5</v>
       </c>
@@ -700,14 +767,17 @@
       <c r="J8" t="s">
         <v>25</v>
       </c>
-      <c r="K8" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="L8" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="M8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>6</v>
       </c>
@@ -726,14 +796,17 @@
       <c r="J9" t="s">
         <v>24</v>
       </c>
-      <c r="K9" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="L9" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>7</v>
       </c>
@@ -755,14 +828,20 @@
       <c r="J10" t="s">
         <v>24</v>
       </c>
-      <c r="K10" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="L10" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N10" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>8</v>
       </c>
@@ -781,14 +860,17 @@
       <c r="J11" t="s">
         <v>24</v>
       </c>
-      <c r="K11" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="L11" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K11" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>9</v>
       </c>
@@ -807,14 +889,20 @@
       <c r="J12" t="s">
         <v>25</v>
       </c>
-      <c r="K12" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="L12" s="12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K12" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="N12" s="13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>10</v>
       </c>
@@ -833,14 +921,20 @@
       <c r="J13" t="s">
         <v>24</v>
       </c>
-      <c r="K13" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="L13" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="K13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="M13" t="s">
+        <v>24</v>
+      </c>
+      <c r="N13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>11</v>
       </c>
@@ -859,16 +953,24 @@
       <c r="J14" t="s">
         <v>25</v>
       </c>
-      <c r="K14" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="L14" s="12" t="s">
+      <c r="K14" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="M14" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="N14" s="13" t="s">
         <v>25</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="B2:H14"/>
-  <mergeCells count="5">
+  <mergeCells count="7">
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="M2:O2"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="B1:C1"/>

</xml_diff>